<commit_message>
sequencer overhaul + ui touchups
</commit_message>
<xml_diff>
--- a/data/character-templates.xlsx
+++ b/data/character-templates.xlsx
@@ -509,36 +509,40 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -797,842 +801,842 @@
   <dimension ref="A1:U1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="10" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="10" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="P2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R2" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="S2" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="T2" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U2" s="3" t="n">
+      <c r="E2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="M2" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="N2" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O2" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R2" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="S2" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="T2" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U2" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="I3" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="L3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="2" t="n">
+      <c r="L3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="P3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R3" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="S3" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="T3" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U3" s="3" t="n">
+      <c r="P3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R3" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="T3" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U3" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="I4" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="K4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="L4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="2" t="n">
+      <c r="L4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="P4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R4" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="S4" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="T4" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U4" s="3" t="n">
+      <c r="P4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="I5" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="L5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="2" t="n">
+      <c r="L5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="P5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R5" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="S5" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="T5" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U5" s="3" t="n">
+      <c r="P5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="S5" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="T5" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U5" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2" t="n">
+      <c r="D6" s="3"/>
+      <c r="E6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G6" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="I6" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="L6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="2" t="n">
+      <c r="L6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="P6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R6" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="S6" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="T6" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U6" s="3" t="n">
+      <c r="P6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="I7" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="L7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="2" t="n">
+      <c r="L7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="P7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R7" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="S7" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="T7" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U7" s="3" t="n">
+      <c r="P7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="S7" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="T7" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U7" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G8" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="I8" s="2" t="n">
+      <c r="I8" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="L8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="2" t="n">
+      <c r="L8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="P8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R8" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="S8" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="T8" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U8" s="3" t="n">
+      <c r="P8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U8" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G9" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="I9" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="K9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="L9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="2" t="n">
+      <c r="L9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="P9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R9" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="S9" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="T9" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U9" s="3" t="n">
+      <c r="P9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R9" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="S9" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="T9" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U9" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="G10" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="I10" s="2" t="n">
+      <c r="I10" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="J10" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="K10" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="L10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="2" t="n">
+      <c r="L10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="P10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R10" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="S10" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="T10" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U10" s="3" t="n">
+      <c r="P10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U10" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F11" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="G11" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="I11" s="2" t="n">
+      <c r="I11" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="J11" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="K11" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="L11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="2" t="n">
+      <c r="L11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="P11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R11" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="S11" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="T11" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U11" s="3" t="n">
+      <c r="P11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R11" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="S11" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="T11" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U11" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2" t="n">
+      <c r="D12" s="3"/>
+      <c r="E12" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="G12" s="3" t="n">
         <v>68</v>
       </c>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="I12" s="2" t="n">
+      <c r="I12" s="3" t="n">
         <v>74</v>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="J12" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K12" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="L12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="2" t="n">
+      <c r="L12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="P12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R12" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="S12" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="T12" s="3" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="U12" s="3" t="n">
+      <c r="P12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R12" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="S12" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="T12" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="U12" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1658,343 +1662,343 @@
   <dimension ref="A1:N9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2" t="n">
+      <c r="G2" s="3"/>
+      <c r="H2" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2" t="n">
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2" t="s">
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2" t="n">
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2" t="s">
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2" t="n">
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="L4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M4" s="2" t="s">
+      <c r="L4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="N4" s="3" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2" t="n">
+      <c r="G5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="L5" s="2" t="n">
+      <c r="L5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="M5" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="N5" s="3" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2" t="n">
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2" t="s">
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2" t="n">
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2" t="s">
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="2" t="n">
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2" t="s">
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="2" t="n">
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2" t="s">
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3" t="s">
         <v>95</v>
       </c>
     </row>
@@ -2017,139 +2021,139 @@
   <dimension ref="A1:B19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="5"/>
+      <c r="B1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="6"/>
+      <c r="A2" s="3"/>
+      <c r="B2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="B3" s="5"/>
+      <c r="B3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2"/>
-      <c r="B9" s="6"/>
+      <c r="A9" s="3"/>
+      <c r="B9" s="7"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="B10" s="5"/>
+      <c r="B10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="7" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2"/>
-      <c r="B17" s="6"/>
+      <c r="A17" s="3"/>
+      <c r="B17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="B18" s="5"/>
+      <c r="B18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="7" t="s">
         <v>122</v>
       </c>
     </row>

</xml_diff>